<commit_message>
Segundo Parcial 18 porcentajes asistencia modificados
</commit_message>
<xml_diff>
--- a/grupos/2AEM - Estadisticos 20222.xlsx
+++ b/grupos/2AEM - Estadisticos 20222.xlsx
@@ -3496,7 +3496,7 @@
         <v>100</v>
       </c>
       <c r="C4">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D4">
         <v>100</v>
@@ -3520,31 +3520,31 @@
         <v>100</v>
       </c>
       <c r="K4">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L4">
         <v>100</v>
       </c>
       <c r="M4">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -3555,7 +3555,7 @@
         <v>100</v>
       </c>
       <c r="C5">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D5">
         <v>100</v>
@@ -3573,37 +3573,37 @@
         <v>100</v>
       </c>
       <c r="I5">
-        <v>90</v>
+        <v>95.5</v>
       </c>
       <c r="J5">
         <v>100</v>
       </c>
       <c r="K5">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L5">
         <v>100</v>
       </c>
       <c r="M5">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>95.5</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -3614,7 +3614,7 @@
         <v>100</v>
       </c>
       <c r="C6">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="D6">
         <v>100</v>
@@ -3629,16 +3629,16 @@
         <v>98.2</v>
       </c>
       <c r="H6">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I6">
-        <v>85</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="J6">
         <v>100</v>
       </c>
       <c r="K6">
-        <v>110</v>
+        <v>95.2</v>
       </c>
       <c r="L6">
         <v>95</v>
@@ -3647,22 +3647,22 @@
         <v>98.2</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -3673,7 +3673,7 @@
         <v>100</v>
       </c>
       <c r="C7">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -3697,7 +3697,7 @@
         <v>100</v>
       </c>
       <c r="K7">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L7">
         <v>100</v>
@@ -3706,22 +3706,22 @@
         <v>100</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -3732,7 +3732,7 @@
         <v>100</v>
       </c>
       <c r="C8">
-        <v>115</v>
+        <v>95.8</v>
       </c>
       <c r="D8">
         <v>100</v>
@@ -3747,40 +3747,40 @@
         <v>100</v>
       </c>
       <c r="H8">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I8">
-        <v>95</v>
+        <v>95.5</v>
       </c>
       <c r="J8">
         <v>100</v>
       </c>
       <c r="K8">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L8">
         <v>100</v>
       </c>
       <c r="M8">
-        <v>96.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>95.5</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S8">
-        <v>0</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -3791,7 +3791,7 @@
         <v>100</v>
       </c>
       <c r="C9">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D9">
         <v>100</v>
@@ -3806,40 +3806,40 @@
         <v>96.40000000000001</v>
       </c>
       <c r="H9">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I9">
-        <v>95</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="J9">
         <v>100</v>
       </c>
       <c r="K9">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L9">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M9">
-        <v>100</v>
+        <v>98.2</v>
       </c>
       <c r="N9">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="P9">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R9">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -3850,7 +3850,7 @@
         <v>83.3</v>
       </c>
       <c r="C10">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D10">
         <v>86.7</v>
@@ -3865,40 +3865,40 @@
         <v>100</v>
       </c>
       <c r="H10">
-        <v>46.7</v>
+        <v>65</v>
       </c>
       <c r="I10">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="J10">
-        <v>73.3</v>
+        <v>80</v>
       </c>
       <c r="K10">
-        <v>30</v>
+        <v>42.9</v>
       </c>
       <c r="L10">
         <v>75</v>
       </c>
       <c r="M10">
+        <v>90</v>
+      </c>
+      <c r="N10">
+        <v>65</v>
+      </c>
+      <c r="O10">
+        <v>75</v>
+      </c>
+      <c r="P10">
         <v>80</v>
       </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
       <c r="Q10">
-        <v>0</v>
+        <v>42.9</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="S10">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -3909,7 +3909,7 @@
         <v>100</v>
       </c>
       <c r="C11">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D11">
         <v>100</v>
@@ -3924,16 +3924,16 @@
         <v>100</v>
       </c>
       <c r="H11">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I11">
-        <v>85</v>
+        <v>93.2</v>
       </c>
       <c r="J11">
         <v>100</v>
       </c>
       <c r="K11">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L11">
         <v>100</v>
@@ -3942,22 +3942,22 @@
         <v>100</v>
       </c>
       <c r="N11">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>93.2</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -3968,7 +3968,7 @@
         <v>93.3</v>
       </c>
       <c r="C12">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D12">
         <v>100</v>
@@ -3983,40 +3983,40 @@
         <v>90.90000000000001</v>
       </c>
       <c r="H12">
-        <v>73.3</v>
+        <v>83.3</v>
       </c>
       <c r="I12">
-        <v>95</v>
+        <v>97.7</v>
       </c>
       <c r="J12">
-        <v>86.7</v>
+        <v>93.3</v>
       </c>
       <c r="K12">
-        <v>90</v>
+        <v>90.5</v>
       </c>
       <c r="L12">
         <v>100</v>
       </c>
       <c r="M12">
-        <v>92.7</v>
+        <v>91.8</v>
       </c>
       <c r="N12">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="O12">
-        <v>0</v>
+        <v>97.7</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>93.3</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>90.5</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S12">
-        <v>0</v>
+        <v>91.8</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -4027,7 +4027,7 @@
         <v>93.3</v>
       </c>
       <c r="C13">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D13">
         <v>100</v>
@@ -4042,40 +4042,40 @@
         <v>89.09999999999999</v>
       </c>
       <c r="H13">
-        <v>46.7</v>
+        <v>70</v>
       </c>
       <c r="I13">
-        <v>55</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="J13">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K13">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="L13">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="M13">
         <v>89.09999999999999</v>
       </c>
       <c r="N13">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -4086,7 +4086,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D14">
         <v>100</v>
@@ -4104,13 +4104,13 @@
         <v>100</v>
       </c>
       <c r="I14">
-        <v>90</v>
+        <v>95.5</v>
       </c>
       <c r="J14">
         <v>100</v>
       </c>
       <c r="K14">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L14">
         <v>100</v>
@@ -4119,22 +4119,22 @@
         <v>100</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>95.5</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S14">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -4145,7 +4145,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>115</v>
+        <v>95.8</v>
       </c>
       <c r="D15">
         <v>100</v>
@@ -4160,40 +4160,40 @@
         <v>92.7</v>
       </c>
       <c r="H15">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I15">
+        <v>93.2</v>
+      </c>
+      <c r="J15">
+        <v>100</v>
+      </c>
+      <c r="K15">
+        <v>95.2</v>
+      </c>
+      <c r="L15">
+        <v>100</v>
+      </c>
+      <c r="M15">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="N15">
         <v>90</v>
       </c>
-      <c r="J15">
-        <v>100</v>
-      </c>
-      <c r="K15">
-        <v>110</v>
-      </c>
-      <c r="L15">
-        <v>100</v>
-      </c>
-      <c r="M15">
-        <v>94.5</v>
-      </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
       <c r="O15">
-        <v>0</v>
+        <v>93.2</v>
       </c>
       <c r="P15">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q15">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S15">
-        <v>0</v>
+        <v>93.59999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -4204,7 +4204,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="D16">
         <v>100</v>
@@ -4219,40 +4219,40 @@
         <v>100</v>
       </c>
       <c r="H16">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I16">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J16">
         <v>100</v>
       </c>
       <c r="K16">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L16">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M16">
         <v>100</v>
       </c>
       <c r="N16">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P16">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q16">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S16">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -4263,7 +4263,7 @@
         <v>93.3</v>
       </c>
       <c r="C17">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D17">
         <v>100</v>
@@ -4278,40 +4278,40 @@
         <v>87.3</v>
       </c>
       <c r="H17">
-        <v>80</v>
+        <v>86.7</v>
       </c>
       <c r="I17">
-        <v>55</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="J17">
         <v>100</v>
       </c>
       <c r="K17">
-        <v>90</v>
+        <v>76.2</v>
       </c>
       <c r="L17">
-        <v>95</v>
+        <v>87.5</v>
       </c>
       <c r="M17">
-        <v>100</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="N17">
-        <v>0</v>
+        <v>86.7</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>76.2</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>87.5</v>
       </c>
       <c r="S17">
-        <v>0</v>
+        <v>93.59999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -4322,7 +4322,7 @@
         <v>96.7</v>
       </c>
       <c r="C18">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D18">
         <v>100</v>
@@ -4337,7 +4337,7 @@
         <v>100</v>
       </c>
       <c r="H18">
-        <v>93.3</v>
+        <v>95</v>
       </c>
       <c r="I18">
         <v>100</v>
@@ -4346,7 +4346,7 @@
         <v>100</v>
       </c>
       <c r="K18">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L18">
         <v>100</v>
@@ -4355,22 +4355,22 @@
         <v>100</v>
       </c>
       <c r="N18">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="O18">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P18">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S18">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -4381,7 +4381,7 @@
         <v>100</v>
       </c>
       <c r="C19">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D19">
         <v>100</v>
@@ -4396,7 +4396,7 @@
         <v>100</v>
       </c>
       <c r="H19">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I19">
         <v>100</v>
@@ -4405,7 +4405,7 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L19">
         <v>100</v>
@@ -4414,22 +4414,22 @@
         <v>100</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O19">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P19">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q19">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S19">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -4440,7 +4440,7 @@
         <v>96.7</v>
       </c>
       <c r="C20">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D20">
         <v>100</v>
@@ -4455,40 +4455,40 @@
         <v>96.40000000000001</v>
       </c>
       <c r="H20">
-        <v>93.3</v>
+        <v>95</v>
       </c>
       <c r="I20">
-        <v>85</v>
+        <v>93.2</v>
       </c>
       <c r="J20">
         <v>100</v>
       </c>
       <c r="K20">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L20">
         <v>100</v>
       </c>
       <c r="M20">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="N20">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="O20">
-        <v>0</v>
+        <v>93.2</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S20">
-        <v>0</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -4499,7 +4499,7 @@
         <v>96.7</v>
       </c>
       <c r="C21">
-        <v>105</v>
+        <v>87.5</v>
       </c>
       <c r="D21">
         <v>100</v>
@@ -4514,40 +4514,40 @@
         <v>90.90000000000001</v>
       </c>
       <c r="H21">
-        <v>86.7</v>
+        <v>91.7</v>
       </c>
       <c r="I21">
-        <v>70</v>
+        <v>79.5</v>
       </c>
       <c r="J21">
         <v>100</v>
       </c>
       <c r="K21">
-        <v>90</v>
+        <v>90.5</v>
       </c>
       <c r="L21">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M21">
-        <v>98.2</v>
+        <v>94.5</v>
       </c>
       <c r="N21">
-        <v>0</v>
+        <v>91.7</v>
       </c>
       <c r="O21">
-        <v>0</v>
+        <v>79.5</v>
       </c>
       <c r="P21">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q21">
-        <v>0</v>
+        <v>90.5</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S21">
-        <v>0</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -4558,7 +4558,7 @@
         <v>93.3</v>
       </c>
       <c r="C22">
-        <v>85</v>
+        <v>70.8</v>
       </c>
       <c r="D22">
         <v>100</v>
@@ -4576,37 +4576,37 @@
         <v>93.3</v>
       </c>
       <c r="I22">
-        <v>50</v>
+        <v>61.4</v>
       </c>
       <c r="J22">
         <v>100</v>
       </c>
       <c r="K22">
-        <v>90</v>
+        <v>76.2</v>
       </c>
       <c r="L22">
-        <v>95</v>
+        <v>82.5</v>
       </c>
       <c r="M22">
-        <v>100</v>
+        <v>95.5</v>
       </c>
       <c r="N22">
-        <v>0</v>
+        <v>93.3</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>61.4</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q22">
-        <v>0</v>
+        <v>76.2</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>82.5</v>
       </c>
       <c r="S22">
-        <v>0</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -4617,7 +4617,7 @@
         <v>93.3</v>
       </c>
       <c r="C23">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D23">
         <v>100</v>
@@ -4632,7 +4632,7 @@
         <v>100</v>
       </c>
       <c r="H23">
-        <v>100</v>
+        <v>96.7</v>
       </c>
       <c r="I23">
         <v>100</v>
@@ -4641,7 +4641,7 @@
         <v>100</v>
       </c>
       <c r="K23">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L23">
         <v>100</v>
@@ -4650,22 +4650,22 @@
         <v>100</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S23">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -4676,7 +4676,7 @@
         <v>96.7</v>
       </c>
       <c r="C24">
-        <v>115</v>
+        <v>95.8</v>
       </c>
       <c r="D24">
         <v>100</v>
@@ -4691,40 +4691,40 @@
         <v>94.5</v>
       </c>
       <c r="H24">
-        <v>80</v>
+        <v>88.3</v>
       </c>
       <c r="I24">
-        <v>55</v>
+        <v>77.3</v>
       </c>
       <c r="J24">
         <v>100</v>
       </c>
       <c r="K24">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L24">
         <v>100</v>
       </c>
       <c r="M24">
-        <v>87.3</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="N24">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>77.3</v>
       </c>
       <c r="P24">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q24">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R24">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S24">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -4735,7 +4735,7 @@
         <v>100</v>
       </c>
       <c r="C25">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D25">
         <v>100</v>
@@ -4750,40 +4750,40 @@
         <v>100</v>
       </c>
       <c r="H25">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I25">
-        <v>80</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J25">
         <v>100</v>
       </c>
       <c r="K25">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L25">
+        <v>95</v>
+      </c>
+      <c r="M25">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="N25">
         <v>90</v>
       </c>
-      <c r="M25">
-        <v>98.2</v>
-      </c>
-      <c r="N25">
-        <v>0</v>
-      </c>
       <c r="O25">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P25">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q25">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="S25">
-        <v>0</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -4794,7 +4794,7 @@
         <v>100</v>
       </c>
       <c r="C26">
-        <v>115</v>
+        <v>95.8</v>
       </c>
       <c r="D26">
         <v>100</v>
@@ -4809,40 +4809,40 @@
         <v>98.2</v>
       </c>
       <c r="H26">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I26">
-        <v>85</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J26">
         <v>100</v>
       </c>
       <c r="K26">
-        <v>100</v>
+        <v>95.2</v>
       </c>
       <c r="L26">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M26">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N26">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O26">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P26">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q26">
-        <v>0</v>
+        <v>95.2</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S26">
-        <v>0</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -4853,7 +4853,7 @@
         <v>100</v>
       </c>
       <c r="C27">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="D27">
         <v>100</v>
@@ -4868,40 +4868,40 @@
         <v>94.5</v>
       </c>
       <c r="H27">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I27">
-        <v>100</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J27">
         <v>100</v>
       </c>
       <c r="K27">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L27">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="M27">
-        <v>100</v>
+        <v>97.3</v>
       </c>
       <c r="N27">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O27">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P27">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q27">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R27">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="S27">
-        <v>0</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="28" spans="1:19">
@@ -4912,7 +4912,7 @@
         <v>100</v>
       </c>
       <c r="C28">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D28">
         <v>100</v>
@@ -4927,40 +4927,40 @@
         <v>98.2</v>
       </c>
       <c r="H28">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I28">
-        <v>80</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J28">
         <v>100</v>
       </c>
       <c r="K28">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L28">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M28">
-        <v>89.09999999999999</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="N28">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O28">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P28">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q28">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R28">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S28">
-        <v>0</v>
+        <v>93.59999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -4971,7 +4971,7 @@
         <v>100</v>
       </c>
       <c r="C29">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D29">
         <v>100</v>
@@ -4989,37 +4989,37 @@
         <v>100</v>
       </c>
       <c r="I29">
-        <v>65</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="J29">
         <v>100</v>
       </c>
       <c r="K29">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L29">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M29">
         <v>98.2</v>
       </c>
       <c r="N29">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O29">
-        <v>0</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="P29">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q29">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R29">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S29">
-        <v>0</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="30" spans="1:19">
@@ -5030,7 +5030,7 @@
         <v>100</v>
       </c>
       <c r="C30">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D30">
         <v>100</v>
@@ -5054,7 +5054,7 @@
         <v>100</v>
       </c>
       <c r="K30">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L30">
         <v>100</v>
@@ -5063,22 +5063,22 @@
         <v>100</v>
       </c>
       <c r="N30">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O30">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P30">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q30">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R30">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S30">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:19">
@@ -5089,7 +5089,7 @@
         <v>100</v>
       </c>
       <c r="C31">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D31">
         <v>100</v>
@@ -5113,7 +5113,7 @@
         <v>100</v>
       </c>
       <c r="K31">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L31">
         <v>100</v>
@@ -5122,22 +5122,22 @@
         <v>100</v>
       </c>
       <c r="N31">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O31">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P31">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q31">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R31">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S31">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:19">
@@ -5148,7 +5148,7 @@
         <v>100</v>
       </c>
       <c r="C32">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D32">
         <v>100</v>
@@ -5163,40 +5163,40 @@
         <v>96.40000000000001</v>
       </c>
       <c r="H32">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I32">
-        <v>80</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J32">
         <v>100</v>
       </c>
       <c r="K32">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L32">
         <v>100</v>
       </c>
       <c r="M32">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="N32">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O32">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P32">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q32">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R32">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S32">
-        <v>0</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="33" spans="1:19">
@@ -5207,7 +5207,7 @@
         <v>100</v>
       </c>
       <c r="C33">
-        <v>105</v>
+        <v>87.5</v>
       </c>
       <c r="D33">
         <v>100</v>
@@ -5222,40 +5222,40 @@
         <v>89.09999999999999</v>
       </c>
       <c r="H33">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I33">
-        <v>90</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="J33">
         <v>100</v>
       </c>
       <c r="K33">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L33">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M33">
-        <v>87.3</v>
+        <v>88.2</v>
       </c>
       <c r="N33">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O33">
-        <v>0</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="P33">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q33">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R33">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S33">
-        <v>0</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="34" spans="1:19">
@@ -5266,7 +5266,7 @@
         <v>100</v>
       </c>
       <c r="C34">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D34">
         <v>100</v>
@@ -5284,37 +5284,37 @@
         <v>100</v>
       </c>
       <c r="I34">
-        <v>95</v>
+        <v>97.7</v>
       </c>
       <c r="J34">
         <v>100</v>
       </c>
       <c r="K34">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L34">
         <v>100</v>
       </c>
       <c r="M34">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N34">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O34">
-        <v>0</v>
+        <v>97.7</v>
       </c>
       <c r="P34">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q34">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R34">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S34">
-        <v>0</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="35" spans="1:19">
@@ -5325,7 +5325,7 @@
         <v>100</v>
       </c>
       <c r="C35">
-        <v>115</v>
+        <v>95.8</v>
       </c>
       <c r="D35">
         <v>100</v>
@@ -5340,16 +5340,16 @@
         <v>100</v>
       </c>
       <c r="H35">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="I35">
-        <v>100</v>
+        <v>97.7</v>
       </c>
       <c r="J35">
         <v>100</v>
       </c>
       <c r="K35">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L35">
         <v>100</v>
@@ -5358,22 +5358,22 @@
         <v>100</v>
       </c>
       <c r="N35">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="O35">
-        <v>0</v>
+        <v>97.7</v>
       </c>
       <c r="P35">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q35">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R35">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S35">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:19">
@@ -5384,7 +5384,7 @@
         <v>80</v>
       </c>
       <c r="C36">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D36">
         <v>100</v>
@@ -5402,37 +5402,37 @@
         <v>80</v>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>81.8</v>
       </c>
       <c r="J36">
         <v>100</v>
       </c>
       <c r="K36">
-        <v>90</v>
+        <v>85.7</v>
       </c>
       <c r="L36">
-        <v>95</v>
+        <v>87.5</v>
       </c>
       <c r="M36">
         <v>85.5</v>
       </c>
       <c r="N36">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="O36">
-        <v>0</v>
+        <v>81.8</v>
       </c>
       <c r="P36">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q36">
-        <v>0</v>
+        <v>85.7</v>
       </c>
       <c r="R36">
-        <v>0</v>
+        <v>87.5</v>
       </c>
       <c r="S36">
-        <v>0</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="37" spans="1:19">
@@ -5443,7 +5443,7 @@
         <v>100</v>
       </c>
       <c r="C37">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D37">
         <v>100</v>
@@ -5458,40 +5458,40 @@
         <v>94.5</v>
       </c>
       <c r="H37">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I37">
-        <v>80</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="J37">
         <v>100</v>
       </c>
       <c r="K37">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L37">
-        <v>95</v>
+        <v>97.5</v>
       </c>
       <c r="M37">
-        <v>89.09999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="N37">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O37">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P37">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q37">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R37">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="S37">
-        <v>0</v>
+        <v>91.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>